<commit_message>
Add Cold/Warm/Closed status tracking to prospect list
Adapted from a cold-call transcript's Cold/Warm/Appointment pipeline
staging, translated to James's actual stack (no GoHighLevel — just the
existing Sheets-based tracker) and his actual sales motion (same-call
close, no separate appointment-booking stage). Replaces the flat
"Contacted?" column with a proper dropdown status.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014CpAYGFcVRHBV6k9TYoyqS
</commit_message>
<xml_diff>
--- a/sales/prospect-list-detailers.xlsx
+++ b/sales/prospect-list-detailers.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Contacted?</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -514,7 +514,11 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -536,7 +540,11 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
@@ -558,7 +566,11 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
@@ -580,7 +592,11 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
@@ -602,7 +618,11 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
@@ -624,7 +644,11 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
@@ -646,7 +670,11 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
@@ -668,7 +696,11 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
@@ -690,7 +722,11 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
@@ -712,7 +748,11 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
@@ -734,7 +774,11 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
@@ -756,7 +800,11 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
@@ -778,7 +826,11 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
@@ -800,7 +852,11 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
@@ -822,7 +878,11 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -844,7 +904,11 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
@@ -866,7 +930,11 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
@@ -888,7 +956,11 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -910,7 +982,11 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
@@ -932,7 +1008,11 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1286,6 +1366,11 @@
       <c r="H56" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid status" error="Pick Cold, Warm, or Closed" type="list">
+      <formula1>"Cold,Warm,Closed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1296,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1399,6 +1484,18 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Status column</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Cold = no contact yet. Warm = a conversation happened, interest is real. Closed = deposit taken. No separate "Appointment" stage — your close happens same-call, not a second booking.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Log first real outreach attempt: In and Out Mobile Detail, no answer
First live call of the LocalPro Labs outreach effort. No answer, follow-up
text sent same day. Status stays Cold pending a real conversation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014CpAYGFcVRHBV6k9TYoyqS
</commit_message>
<xml_diff>
--- a/sales/prospect-list-detailers.xlsx
+++ b/sales/prospect-list-detailers.xlsx
@@ -519,7 +519,11 @@
           <t>Cold</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Called 9/11, no answer. Sent follow-up text same day. Retry or wait for reply.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>